<commit_message>
fix: load master list dropdown options dynamically from database and clear database on sync
</commit_message>
<xml_diff>
--- a/Mã Bun.xlsx
+++ b/Mã Bun.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv2_ortholite_vn/Documents/PROJECT LÂM/DailyFoamingReport/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="8_{4BBF591A-BB74-4A17-8CD8-3CE44677F576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6389C5F2-CF70-4596-AB54-89BE1539BCD3}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="8_{4BBF591A-BB74-4A17-8CD8-3CE44677F576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D5692F0-B78A-400C-9BC0-F46841932ECA}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{89885EAB-F083-429F-A501-EC1C8FB42915}"/>
   </bookViews>
@@ -4233,33 +4233,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CFE8195C-E963-48E9-8AB5-525E9503C127}" name="Table1" displayName="Table1" ref="A1:L458" totalsRowShown="0" headerRowDxfId="30" dataDxfId="28" headerRowBorderDxfId="29" tableBorderDxfId="27" totalsRowBorderDxfId="26">
-  <autoFilter ref="A1:L458" xr:uid="{CFE8195C-E963-48E9-8AB5-525E9503C127}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="YELLOW"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="6">
-      <filters>
-        <filter val="0.11D"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="7">
-      <filters>
-        <filter val="25C"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="8">
-      <filters>
-        <filter val="CSĐ"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="9">
-      <filters>
-        <filter val="2.00M"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:L458" xr:uid="{CFE8195C-E963-48E9-8AB5-525E9503C127}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L404">
     <sortCondition ref="L1:L457"/>
   </sortState>
@@ -4599,7 +4573,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="str">
         <f t="shared" ref="A2:A65" si="0">RIGHT(B2,3)</f>
         <v>190</v>
@@ -4635,7 +4609,7 @@
         <v>Ultra  0.085D - 15C - CSĐ   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="3" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="str">
         <f t="shared" si="0"/>
         <v>074</v>
@@ -4671,7 +4645,7 @@
         <v>Ultra  0.085D - 15C - CSĐ   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="4" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="str">
         <f t="shared" si="0"/>
         <v>072</v>
@@ -4707,7 +4681,7 @@
         <v>Ultra  0.085D - 15C - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="5" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="str">
         <f t="shared" si="0"/>
         <v>063</v>
@@ -4743,7 +4717,7 @@
         <v>Ultra  0.085D - 15C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="6" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="str">
         <f t="shared" si="0"/>
         <v>349</v>
@@ -4783,7 +4757,7 @@
         <v>Ultra  0.085D - 15C - CSĐ   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="str">
         <f t="shared" si="0"/>
         <v>108</v>
@@ -4819,7 +4793,7 @@
         <v>EcoLT  0.085D - 15C - CSĐ HB   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="str">
         <f t="shared" si="0"/>
         <v>110</v>
@@ -4855,7 +4829,7 @@
         <v>EcoLT  0.085D - 15C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="9" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="str">
         <f t="shared" si="0"/>
         <v>364</v>
@@ -4891,7 +4865,7 @@
         <v>Ultra  0.085D - 15C - CSĐ HB   /   NEUTRAL GRAY - 2.00M</v>
       </c>
     </row>
-    <row r="10" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="str">
         <f t="shared" si="0"/>
         <v>297</v>
@@ -4927,7 +4901,7 @@
         <v>Ultra  0.085D - 15C - CSĐ HB   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="11" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="str">
         <f t="shared" si="0"/>
         <v>194</v>
@@ -4963,7 +4937,7 @@
         <v>Ultra  0.085D - 15C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="12" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="str">
         <f t="shared" si="0"/>
         <v>166</v>
@@ -4999,7 +4973,7 @@
         <v>Ultra  0.085D - 15C - NIKE   /   LIME GREEN -  1.7M</v>
       </c>
     </row>
-    <row r="13" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="str">
         <f t="shared" si="0"/>
         <v>165</v>
@@ -5039,7 +5013,7 @@
         <v>Ultra  0.085D - 15C - Nike   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="14" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="str">
         <f t="shared" si="0"/>
         <v>158</v>
@@ -5079,7 +5053,7 @@
         <v>Ultra  0.085D - 15C - Nike   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="str">
         <f t="shared" si="0"/>
         <v>177</v>
@@ -5115,7 +5089,7 @@
         <v>Ultra  0.085D - 15C - NIKE HB   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="16" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="str">
         <f t="shared" si="0"/>
         <v>171</v>
@@ -5151,7 +5125,7 @@
         <v>Ultra  0.085D - 15C - NIKE HB   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="17" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="str">
         <f t="shared" si="0"/>
         <v>173</v>
@@ -5187,7 +5161,7 @@
         <v>Ultra  0.085D - 15C - NIKE HB   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="18" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="str">
         <f t="shared" si="0"/>
         <v>169</v>
@@ -5223,7 +5197,7 @@
         <v>Ultra  0.085D - 15C - NIKE HB   /   NEUTRAL GRAY - 2.00M</v>
       </c>
     </row>
-    <row r="19" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="str">
         <f t="shared" si="0"/>
         <v>170</v>
@@ -5259,7 +5233,7 @@
         <v>Ultra  0.085D - 15C - NIKE HB   /   RED - 2.00M</v>
       </c>
     </row>
-    <row r="20" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="str">
         <f t="shared" si="0"/>
         <v>174</v>
@@ -5299,7 +5273,7 @@
         <v>Ultra  0.085D - 15C - Nike HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="21" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="str">
         <f t="shared" si="0"/>
         <v>356</v>
@@ -5339,7 +5313,7 @@
         <v>EcoLT  0.11D - 15C - CSĐ   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="22" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="str">
         <f t="shared" si="0"/>
         <v>075</v>
@@ -5375,7 +5349,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   AIR BLUE - 1.47M</v>
       </c>
     </row>
-    <row r="23" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="str">
         <f t="shared" si="0"/>
         <v>001</v>
@@ -5411,7 +5385,7 @@
         <v>Regular  0.11D - 15C - CSĐ   /   BURNT SIENNA - 2.00M</v>
       </c>
     </row>
-    <row r="24" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="str">
         <f t="shared" si="0"/>
         <v>022</v>
@@ -5447,7 +5421,7 @@
         <v>Regular  0.11D - 15C - CSĐ   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="25" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="str">
         <f t="shared" si="0"/>
         <v>027</v>
@@ -5483,7 +5457,7 @@
         <v>Regular  0.11D - 15C - CSĐ   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="26" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="str">
         <f t="shared" si="0"/>
         <v>049</v>
@@ -5519,7 +5493,7 @@
         <v>Regular  0.11D - 15C - CSĐ   /   TRUE BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="27" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="str">
         <f t="shared" si="0"/>
         <v>002</v>
@@ -5559,7 +5533,7 @@
         <v>Regular  0.11D - 15C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="28" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="str">
         <f t="shared" si="0"/>
         <v>311</v>
@@ -5595,7 +5569,7 @@
         <v>Regular  0.11D - 15C - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="29" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="str">
         <f t="shared" si="0"/>
         <v>377</v>
@@ -5631,7 +5605,7 @@
         <v>Regular  0.11D - 15C - CSĐ   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="30" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="str">
         <f t="shared" si="0"/>
         <v>071</v>
@@ -5667,7 +5641,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="31" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="str">
         <f t="shared" si="0"/>
         <v>017</v>
@@ -5703,7 +5677,7 @@
         <v>Regular  0.11D - 15C - CSĐ   /   YELLOW -  1.7M</v>
       </c>
     </row>
-    <row r="32" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="str">
         <f t="shared" si="0"/>
         <v>111</v>
@@ -5739,7 +5713,7 @@
         <v>EcoLT  0.11D - 15C - CSĐ HB   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="33" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="str">
         <f t="shared" si="0"/>
         <v>360</v>
@@ -5775,7 +5749,7 @@
         <v>EcoLT  0.11D - 15C - CSĐ HB   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="34" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="str">
         <f t="shared" si="0"/>
         <v>283</v>
@@ -5811,7 +5785,7 @@
         <v>Regular  0.11D - 15C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="35" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="str">
         <f t="shared" si="0"/>
         <v>127</v>
@@ -5847,7 +5821,7 @@
         <v>Regular  0.11D - 15C - NIKE   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="36" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="str">
         <f t="shared" si="0"/>
         <v>122</v>
@@ -5883,7 +5857,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="str">
         <f t="shared" si="0"/>
         <v>263</v>
@@ -5919,7 +5893,7 @@
         <v>Regular  0.13D - 15C - CSĐ   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="38" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="str">
         <f t="shared" si="0"/>
         <v>359</v>
@@ -5955,7 +5929,7 @@
         <v>Regular  0.13D - 15C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="str">
         <f t="shared" si="0"/>
         <v>317</v>
@@ -5995,7 +5969,7 @@
         <v>Regular  0.13D - 15C - CSĐ   /   NEUTRAL GRAY - 2.00M</v>
       </c>
     </row>
-    <row r="40" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="str">
         <f t="shared" si="0"/>
         <v>034</v>
@@ -6031,7 +6005,7 @@
         <v>Regular  0.13D - 15C - CSĐ   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="41" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="str">
         <f t="shared" si="0"/>
         <v>224</v>
@@ -6071,7 +6045,7 @@
         <v>R&amp;R  0.16D - 15C - CSĐ   /   CASTLEROCK - 1.7M</v>
       </c>
     </row>
-    <row r="42" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="str">
         <f t="shared" si="0"/>
         <v>267</v>
@@ -6107,7 +6081,7 @@
         <v>R&amp;R  0.16D - 15C - CSĐ   /   SEEDPEARL -  1.7M</v>
       </c>
     </row>
-    <row r="43" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="str">
         <f t="shared" si="0"/>
         <v>219</v>
@@ -6143,7 +6117,7 @@
         <v>Float  0.185D - 15C - CSĐ   /   BLUE ATOLL -  1.7M</v>
       </c>
     </row>
-    <row r="44" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="str">
         <f t="shared" si="0"/>
         <v>076</v>
@@ -6183,7 +6157,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   BILLIARD - 2.00M</v>
       </c>
     </row>
-    <row r="45" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="str">
         <f t="shared" si="0"/>
         <v>345</v>
@@ -6219,7 +6193,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   BROWN SUGAR - 2.00M</v>
       </c>
     </row>
-    <row r="46" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="str">
         <f t="shared" si="0"/>
         <v>358</v>
@@ -6255,7 +6229,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   FOSSIL - 2.00M</v>
       </c>
     </row>
-    <row r="47" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="str">
         <f t="shared" si="0"/>
         <v>220</v>
@@ -6291,7 +6265,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   BILLIARD - 1.47M</v>
       </c>
     </row>
-    <row r="48" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="str">
         <f t="shared" si="0"/>
         <v>168</v>
@@ -6327,7 +6301,7 @@
         <v>Ultra  0.085D - 25C - NIKE   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="49" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="str">
         <f t="shared" si="0"/>
         <v>083</v>
@@ -6367,7 +6341,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ   /   300C - 2.00M</v>
       </c>
     </row>
-    <row r="50" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="str">
         <f t="shared" si="0"/>
         <v>083</v>
@@ -6407,7 +6381,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ   /   300C - 2.00M</v>
       </c>
     </row>
-    <row r="51" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="str">
         <f t="shared" si="0"/>
         <v>107</v>
@@ -6447,7 +6421,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ HB   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="52" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="str">
         <f t="shared" si="0"/>
         <v>207</v>
@@ -6483,7 +6457,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ HB   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="53" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="str">
         <f t="shared" si="0"/>
         <v>097</v>
@@ -6523,7 +6497,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="54" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="str">
         <f t="shared" si="0"/>
         <v>097</v>
@@ -6563,7 +6537,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="55" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="str">
         <f t="shared" si="0"/>
         <v>332</v>
@@ -6603,7 +6577,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   CASTLEROCK - 2.00M</v>
       </c>
     </row>
-    <row r="56" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="str">
         <f t="shared" si="0"/>
         <v>341</v>
@@ -6643,7 +6617,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="57" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="str">
         <f t="shared" si="0"/>
         <v>344</v>
@@ -6683,7 +6657,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="58" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="str">
         <f t="shared" si="0"/>
         <v>342</v>
@@ -6723,7 +6697,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   NEUTRAL GRAY - 2.00M</v>
       </c>
     </row>
-    <row r="59" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="str">
         <f t="shared" si="0"/>
         <v>097</v>
@@ -6763,7 +6737,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="60" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A60" s="5" t="str">
         <f t="shared" si="0"/>
         <v>181</v>
@@ -6803,7 +6777,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="61" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="str">
         <f t="shared" si="0"/>
         <v>276</v>
@@ -6839,7 +6813,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   BILLIARD -  1.7M</v>
       </c>
     </row>
-    <row r="62" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="str">
         <f t="shared" si="0"/>
         <v>213</v>
@@ -6879,7 +6853,7 @@
         <v>X-25  0.12D - 20C - CSĐ HB   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="63" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="str">
         <f t="shared" si="0"/>
         <v>109</v>
@@ -6915,7 +6889,7 @@
         <v>EcoLT  0.13D - 25C - CSĐ HB   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="64" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A64" s="5" t="str">
         <f t="shared" si="0"/>
         <v>189</v>
@@ -6951,7 +6925,7 @@
         <v>EcoLT  0.13D - 25C - CSĐ HB   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="65" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="str">
         <f t="shared" si="0"/>
         <v>321</v>
@@ -6991,7 +6965,7 @@
         <v>Float  0.12D - 21C - CSĐ   /   BLUE ATOLL - 2.00M</v>
       </c>
     </row>
-    <row r="66" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A66" s="5" t="str">
         <f t="shared" ref="A66:A129" si="1">RIGHT(B66,3)</f>
         <v>321</v>
@@ -7031,7 +7005,7 @@
         <v>Float  0.12D - 21C - CSĐ   /   BLUE ATOLL - 2.00M</v>
       </c>
     </row>
-    <row r="67" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A67" s="5" t="str">
         <f t="shared" si="1"/>
         <v>375</v>
@@ -7067,7 +7041,7 @@
         <v>X-25  0.12D - 20C - NIKE   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="68" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="str">
         <f t="shared" si="1"/>
         <v>373</v>
@@ -7107,7 +7081,7 @@
         <v>X-25  0.12D - 20C - Nike   /   BILLIARD - 2.00M</v>
       </c>
     </row>
-    <row r="69" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A69" s="5" t="str">
         <f t="shared" si="1"/>
         <v>339</v>
@@ -7147,7 +7121,7 @@
         <v>Float  0.12D - 21C - CSĐ   /   NEUTRAL GRAY - 2.00M</v>
       </c>
     </row>
-    <row r="70" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A70" s="5" t="str">
         <f t="shared" si="1"/>
         <v>339</v>
@@ -7187,7 +7161,7 @@
         <v>Float  0.12D - 21C - CSĐ   /   NEUTRAL GRAY - 2.00M</v>
       </c>
     </row>
-    <row r="71" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A71" s="5" t="str">
         <f t="shared" si="1"/>
         <v>346</v>
@@ -7227,7 +7201,7 @@
         <v>Float  0.12D - 21C - CSĐ   /   NEUTRAL GRAY - 1.47M</v>
       </c>
     </row>
-    <row r="72" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="str">
         <f t="shared" si="1"/>
         <v>209</v>
@@ -7267,7 +7241,7 @@
         <v>HybridPlus  0.12D - 25C - CSĐ HB   /   MINT GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="73" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="str">
         <f t="shared" si="1"/>
         <v>209</v>
@@ -7307,7 +7281,7 @@
         <v>HybridPlus  0.12D - 25C - CSĐ HB   /   MINT GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="74" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A74" s="5" t="str">
         <f t="shared" si="1"/>
         <v>340</v>
@@ -7347,7 +7321,7 @@
         <v>Float  0.12D - 21C - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="75" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A75" s="5" t="str">
         <f t="shared" si="1"/>
         <v>352</v>
@@ -7383,7 +7357,7 @@
         <v>Float  0.12D - 21C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="76" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="str">
         <f t="shared" si="1"/>
         <v>089</v>
@@ -7419,7 +7393,7 @@
         <v>EcoLT  0.085D - 25C - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="77" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A77" s="5" t="str">
         <f t="shared" si="1"/>
         <v>057</v>
@@ -7459,7 +7433,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="78" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A78" s="5" t="str">
         <f t="shared" si="1"/>
         <v>058</v>
@@ -7499,7 +7473,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="79" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="str">
         <f t="shared" si="1"/>
         <v>272</v>
@@ -7535,7 +7509,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   BLACK - 2.00M</v>
       </c>
     </row>
-    <row r="80" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A80" s="5" t="str">
         <f t="shared" si="1"/>
         <v>060</v>
@@ -7571,7 +7545,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   BURNT SIENNA - 2.00M</v>
       </c>
     </row>
-    <row r="81" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A81" s="5" t="str">
         <f t="shared" si="1"/>
         <v>065</v>
@@ -7607,7 +7581,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   FOSSIL - 2.00M</v>
       </c>
     </row>
-    <row r="82" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A82" s="5" t="str">
         <f t="shared" si="1"/>
         <v>066</v>
@@ -7643,7 +7617,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="83" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A83" s="5" t="str">
         <f t="shared" si="1"/>
         <v>062</v>
@@ -7679,7 +7653,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="84" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A84" s="5" t="str">
         <f t="shared" si="1"/>
         <v>073</v>
@@ -7715,7 +7689,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   NEUTRAL GRAY - 2.00M</v>
       </c>
     </row>
-    <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A85" s="5" t="str">
         <f t="shared" si="1"/>
         <v>294</v>
@@ -7751,7 +7725,7 @@
         <v>Ultra  0.085D - 5-10C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="86" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A86" s="5" t="str">
         <f t="shared" si="1"/>
         <v>059</v>
@@ -7787,7 +7761,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   RED - 2.00M</v>
       </c>
     </row>
-    <row r="87" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A87" s="5" t="str">
         <f t="shared" si="1"/>
         <v>036</v>
@@ -7823,7 +7797,7 @@
         <v>Regular  0.11D - 15C - CSĐ   /   AIR BLUE -  1.7M</v>
       </c>
     </row>
-    <row r="88" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A88" s="5" t="str">
         <f t="shared" si="1"/>
         <v>064</v>
@@ -7859,7 +7833,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   GREEN - 1.47M</v>
       </c>
     </row>
-    <row r="89" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A89" s="5" t="str">
         <f t="shared" si="1"/>
         <v>068</v>
@@ -7895,7 +7869,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   GREY - 1.47M</v>
       </c>
     </row>
-    <row r="90" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A90" s="5" t="str">
         <f t="shared" si="1"/>
         <v>069</v>
@@ -7931,7 +7905,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   RED - 1.47M</v>
       </c>
     </row>
-    <row r="91" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A91" s="5" t="str">
         <f t="shared" si="1"/>
         <v>061</v>
@@ -7967,7 +7941,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="92" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A92" s="5" t="str">
         <f t="shared" si="1"/>
         <v>209</v>
@@ -8007,7 +7981,7 @@
         <v>HybridPlus  0.12D - 25C - CSĐ HB   /   MINT GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="93" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A93" s="5" t="str">
         <f t="shared" si="1"/>
         <v>348</v>
@@ -8047,7 +8021,7 @@
         <v>Imperial  0.22D - 25C - CSĐ   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="94" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A94" s="5" t="str">
         <f t="shared" si="1"/>
         <v>348</v>
@@ -8087,7 +8061,7 @@
         <v>Imperial  0.22D - 25C - CSĐ   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="95" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A95" s="5" t="str">
         <f t="shared" si="1"/>
         <v>010</v>
@@ -8127,7 +8101,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="96" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A96" s="5" t="str">
         <f t="shared" si="1"/>
         <v>264</v>
@@ -8167,7 +8141,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   YELLOW - 1.47M</v>
       </c>
     </row>
-    <row r="97" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A97" s="5" t="str">
         <f t="shared" si="1"/>
         <v>010</v>
@@ -8207,7 +8181,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="98" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A98" s="5" t="str">
         <f t="shared" si="1"/>
         <v>010</v>
@@ -8247,7 +8221,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="99" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A99" s="5" t="str">
         <f t="shared" si="1"/>
         <v>004</v>
@@ -8287,7 +8261,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="100" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A100" s="5" t="str">
         <f t="shared" si="1"/>
         <v>004</v>
@@ -8327,7 +8301,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="101" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A101" s="5" t="str">
         <f t="shared" si="1"/>
         <v>070</v>
@@ -8363,7 +8337,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   RED -  1.7M</v>
       </c>
     </row>
-    <row r="102" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A102" s="5" t="str">
         <f t="shared" si="1"/>
         <v>103</v>
@@ -8399,7 +8373,7 @@
         <v>EcoLT  0.085D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="103" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A103" s="5" t="str">
         <f t="shared" si="1"/>
         <v>104</v>
@@ -8435,7 +8409,7 @@
         <v>EcoLT  0.085D - 25C - CSĐ HB   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="104" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A104" s="5" t="str">
         <f t="shared" si="1"/>
         <v>004</v>
@@ -8475,7 +8449,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="105" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A105" s="5" t="str">
         <f t="shared" si="1"/>
         <v>239</v>
@@ -8511,7 +8485,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   BLACK - 2.00M</v>
       </c>
     </row>
-    <row r="106" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A106" s="5" t="str">
         <f t="shared" si="1"/>
         <v>243</v>
@@ -8547,7 +8521,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="107" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A107" s="5" t="str">
         <f t="shared" si="1"/>
         <v>121</v>
@@ -8583,7 +8557,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="108" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A108" s="5" t="str">
         <f t="shared" si="1"/>
         <v>265</v>
@@ -8619,7 +8593,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   NINE IRON - 2.00M</v>
       </c>
     </row>
-    <row r="109" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A109" s="5" t="str">
         <f t="shared" si="1"/>
         <v>008</v>
@@ -8659,7 +8633,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="110" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A110" s="5" t="str">
         <f t="shared" si="1"/>
         <v>124</v>
@@ -8695,7 +8669,7 @@
         <v xml:space="preserve">Ultra  0.085D - 25C - CSĐ HB   /   SEEDPEARL - 1.47M </v>
       </c>
     </row>
-    <row r="111" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A111" s="5" t="str">
         <f t="shared" si="1"/>
         <v>119</v>
@@ -8731,7 +8705,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="112" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A112" s="5" t="str">
         <f t="shared" si="1"/>
         <v>009</v>
@@ -8767,7 +8741,7 @@
         <v>Regular  0.11D - 15C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="113" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A113" s="5" t="str">
         <f t="shared" si="1"/>
         <v>193</v>
@@ -8803,7 +8777,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   SEEDPEARL -  1.7M</v>
       </c>
     </row>
-    <row r="114" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A114" s="5" t="str">
         <f t="shared" si="1"/>
         <v>008</v>
@@ -8843,7 +8817,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="115" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A115" s="5" t="str">
         <f t="shared" si="1"/>
         <v>113</v>
@@ -8883,7 +8857,7 @@
         <v>Regular  0.11D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="116" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A116" s="5" t="str">
         <f t="shared" si="1"/>
         <v>113</v>
@@ -8923,7 +8897,7 @@
         <v>Regular  0.11D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="117" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A117" s="5" t="str">
         <f t="shared" si="1"/>
         <v>188</v>
@@ -8963,7 +8937,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="118" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A118" s="5" t="str">
         <f t="shared" si="1"/>
         <v>113</v>
@@ -9003,7 +8977,7 @@
         <v>Regular  0.11D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="119" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A119" s="5" t="str">
         <f t="shared" si="1"/>
         <v>113</v>
@@ -9043,7 +9017,7 @@
         <v>Regular  0.11D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="120" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A120" s="5" t="str">
         <f t="shared" si="1"/>
         <v>113</v>
@@ -9083,7 +9057,7 @@
         <v>Regular  0.11D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="121" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A121" s="5" t="str">
         <f t="shared" si="1"/>
         <v>113</v>
@@ -9123,7 +9097,7 @@
         <v>Regular  0.11D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="122" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A122" s="5" t="str">
         <f t="shared" si="1"/>
         <v>137</v>
@@ -9163,7 +9137,7 @@
         <v>Regular  0.11D - 25C - Nike   /   AIR BLUE - 1.47M</v>
       </c>
     </row>
-    <row r="123" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A123" s="5" t="str">
         <f t="shared" si="1"/>
         <v>232</v>
@@ -9199,7 +9173,7 @@
         <v>Regular  0.11D - 25C - NIKE   /   AIR BLUE - 1.47M</v>
       </c>
     </row>
-    <row r="124" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A124" s="5" t="str">
         <f t="shared" si="1"/>
         <v>164</v>
@@ -9239,7 +9213,7 @@
         <v>Ultra  0.085D - 25C - Nike   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="125" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A125" s="5" t="str">
         <f t="shared" si="1"/>
         <v>300</v>
@@ -9279,7 +9253,7 @@
         <v>Ultra  0.085D - 25C - Nike   /   SEEDPEARL - 1.70M</v>
       </c>
     </row>
-    <row r="126" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A126" s="5" t="str">
         <f t="shared" si="1"/>
         <v>131</v>
@@ -9319,7 +9293,7 @@
         <v>Regular  0.11D - 15C - Nike   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="127" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A127" s="5" t="str">
         <f t="shared" si="1"/>
         <v>159</v>
@@ -9355,7 +9329,7 @@
         <v>Ultra  0.085D - 25C - NIKE   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="128" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A128" s="5" t="str">
         <f t="shared" si="1"/>
         <v>195</v>
@@ -9391,7 +9365,7 @@
         <v>Ultra  0.085D - 25C - NIKE   /   GREY -  1.7M</v>
       </c>
     </row>
-    <row r="129" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A129" s="5" t="str">
         <f t="shared" si="1"/>
         <v>167</v>
@@ -9427,7 +9401,7 @@
         <v>Ultra  0.085D - 25C - NIKE   /   LIME GREEN -  1.7M</v>
       </c>
     </row>
-    <row r="130" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A130" s="5" t="str">
         <f t="shared" ref="A130:A193" si="2">RIGHT(B130,3)</f>
         <v>161</v>
@@ -9467,7 +9441,7 @@
         <v>Ultra  0.085D - 25C - Nike   /   FOSSIL - 2.00M</v>
       </c>
     </row>
-    <row r="131" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A131" s="5" t="str">
         <f t="shared" si="2"/>
         <v>164</v>
@@ -9507,7 +9481,7 @@
         <v>Ultra  0.085D - 25C - Nike   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="132" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A132" s="5" t="str">
         <f t="shared" si="2"/>
         <v>160</v>
@@ -9547,7 +9521,7 @@
         <v>Ultra  0.085D - 25C - Nike   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="133" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A133" s="5" t="str">
         <f t="shared" si="2"/>
         <v>162</v>
@@ -9587,7 +9561,7 @@
         <v>Ultra  0.085D - 25C - Nike   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="134" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A134" s="5" t="str">
         <f t="shared" si="2"/>
         <v>163</v>
@@ -9627,7 +9601,7 @@
         <v>Ultra  0.085D - 25C - Nike   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="135" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A135" s="5" t="str">
         <f t="shared" si="2"/>
         <v>172</v>
@@ -9663,7 +9637,7 @@
         <v>Ultra  0.085D - 25C - NIKE HB   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="136" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A136" s="5" t="str">
         <f t="shared" si="2"/>
         <v>176</v>
@@ -9699,7 +9673,7 @@
         <v>Ultra  0.085D - 25C - NIKE HB   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="137" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A137" s="5" t="str">
         <f t="shared" si="2"/>
         <v>178</v>
@@ -9735,7 +9709,7 @@
         <v>Ultra  0.085D - 25C - NIKE HB   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="138" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A138" s="5" t="str">
         <f t="shared" si="2"/>
         <v>125</v>
@@ -9775,7 +9749,7 @@
         <v>Regular  0.11D - 25C - Nike   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="139" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A139" s="5" t="str">
         <f t="shared" si="2"/>
         <v>125</v>
@@ -9815,7 +9789,7 @@
         <v>Regular  0.11D - 25C - Nike   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="140" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A140" s="5" t="str">
         <f t="shared" si="2"/>
         <v>094</v>
@@ -9855,7 +9829,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ   /   300C - 1.47M</v>
       </c>
     </row>
-    <row r="141" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A141" s="5" t="str">
         <f t="shared" si="2"/>
         <v>125</v>
@@ -9895,7 +9869,7 @@
         <v>Regular  0.11D - 25C - Nike   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="142" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A142" s="5" t="str">
         <f t="shared" si="2"/>
         <v>149</v>
@@ -9935,7 +9909,7 @@
         <v>Regular  0.11D - 25C - Nike HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="143" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A143" s="5" t="str">
         <f t="shared" si="2"/>
         <v>085</v>
@@ -10015,7 +9989,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="145" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A145" s="5" t="str">
         <f t="shared" si="2"/>
         <v>023</v>
@@ -10051,7 +10025,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   AIR BLUE -  1.7M</v>
       </c>
     </row>
-    <row r="146" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A146" s="11" t="str">
         <f t="shared" si="2"/>
         <v>191</v>
@@ -10087,7 +10061,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ   /   FOSSIL - 2.00M</v>
       </c>
     </row>
-    <row r="147" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A147" s="11" t="str">
         <f t="shared" si="2"/>
         <v>087</v>
@@ -10123,7 +10097,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="148" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A148" s="11" t="str">
         <f t="shared" si="2"/>
         <v>096</v>
@@ -10159,7 +10133,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="149" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A149" s="11" t="str">
         <f t="shared" si="2"/>
         <v>187</v>
@@ -10195,7 +10169,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ   /   NEUTRAL GRAY - 2.00M</v>
       </c>
     </row>
-    <row r="150" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A150" s="11" t="str">
         <f t="shared" si="2"/>
         <v>088</v>
@@ -10231,7 +10205,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ   /   RED - 2.00M</v>
       </c>
     </row>
-    <row r="151" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A151" s="11" t="str">
         <f t="shared" si="2"/>
         <v>095</v>
@@ -10267,7 +10241,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ   /   300C -  1.7M</v>
       </c>
     </row>
-    <row r="152" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A152" s="5" t="str">
         <f t="shared" si="2"/>
         <v>025</v>
@@ -10307,7 +10281,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="153" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A153" s="11" t="str">
         <f t="shared" si="2"/>
         <v>379</v>
@@ -10343,7 +10317,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   BROWN SUGAR - 2.00M</v>
       </c>
     </row>
-    <row r="154" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A154" s="11" t="str">
         <f t="shared" si="2"/>
         <v>007</v>
@@ -10379,7 +10353,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   AMAZON - 2.00M</v>
       </c>
     </row>
-    <row r="155" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A155" s="11" t="str">
         <f t="shared" si="2"/>
         <v>019</v>
@@ -10451,7 +10425,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="157" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A157" s="11" t="str">
         <f t="shared" si="2"/>
         <v>014</v>
@@ -10487,7 +10461,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   AIR BLUE - 1.47M</v>
       </c>
     </row>
-    <row r="158" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A158" s="11" t="str">
         <f t="shared" si="2"/>
         <v>093</v>
@@ -10523,7 +10497,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="159" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A159" s="11" t="str">
         <f t="shared" si="2"/>
         <v>149</v>
@@ -10563,7 +10537,7 @@
         <v>Regular  0.11D - 25C - Nike HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="160" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A160" s="11" t="str">
         <f t="shared" si="2"/>
         <v>031</v>
@@ -10599,7 +10573,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   BURNT SIENNA - 2.00M</v>
       </c>
     </row>
-    <row r="161" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A161" s="11" t="str">
         <f t="shared" si="2"/>
         <v>011</v>
@@ -10639,7 +10613,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="162" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A162" s="5" t="str">
         <f t="shared" si="2"/>
         <v>011</v>
@@ -10679,7 +10653,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="163" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A163" s="11" t="str">
         <f t="shared" si="2"/>
         <v>011</v>
@@ -10719,7 +10693,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="164" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A164" s="11" t="str">
         <f t="shared" si="2"/>
         <v>011</v>
@@ -10759,7 +10733,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="165" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A165" s="11" t="str">
         <f t="shared" si="2"/>
         <v>011</v>
@@ -10799,7 +10773,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="166" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A166" s="11" t="str">
         <f t="shared" si="2"/>
         <v>039</v>
@@ -10839,7 +10813,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   NEUTRAL GRAY - 2.00M</v>
       </c>
     </row>
-    <row r="167" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A167" s="11" t="str">
         <f t="shared" si="2"/>
         <v>032</v>
@@ -10879,7 +10853,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="168" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A168" s="5" t="str">
         <f t="shared" si="2"/>
         <v>011</v>
@@ -10919,7 +10893,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="169" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A169" s="11" t="str">
         <f t="shared" si="2"/>
         <v>006</v>
@@ -10955,7 +10929,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   GREY - 1.47M</v>
       </c>
     </row>
-    <row r="170" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A170" s="11" t="str">
         <f t="shared" si="2"/>
         <v>184</v>
@@ -10991,7 +10965,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   NEUTRAL GRAY - 1.47M</v>
       </c>
     </row>
-    <row r="171" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A171" s="11" t="str">
         <f t="shared" si="2"/>
         <v>030</v>
@@ -11027,7 +11001,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   RED - 1.47M</v>
       </c>
     </row>
-    <row r="172" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A172" s="11" t="str">
         <f t="shared" si="2"/>
         <v>387</v>
@@ -11065,7 +11039,7 @@
         <v>Regular  0.16D - 51C - CSĐ   /   AMAZON - 1.7M</v>
       </c>
     </row>
-    <row r="173" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A173" s="11" t="str">
         <f t="shared" si="2"/>
         <v>045</v>
@@ -11101,7 +11075,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   GREEN -  1.7M</v>
       </c>
     </row>
-    <row r="174" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A174" s="11" t="str">
         <f t="shared" si="2"/>
         <v>024</v>
@@ -11137,7 +11111,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   GREY -  1.7M</v>
       </c>
     </row>
-    <row r="175" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A175" s="11" t="str">
         <f t="shared" si="2"/>
         <v>050</v>
@@ -11173,7 +11147,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   NEUTRAL GRAY -  1.7M</v>
       </c>
     </row>
-    <row r="176" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A176" s="11" t="str">
         <f t="shared" si="2"/>
         <v>038</v>
@@ -11209,7 +11183,7 @@
         <v>Regular  0.11D - 25C - CSĐ   /   YELLOW -  1.7M</v>
       </c>
     </row>
-    <row r="177" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A177" s="11" t="str">
         <f t="shared" si="2"/>
         <v>376</v>
@@ -11245,7 +11219,7 @@
         <v>Regular   0.11D - 25C - CSĐ   /   BLACK - 2.00M</v>
       </c>
     </row>
-    <row r="178" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A178" s="11" t="str">
         <f t="shared" si="2"/>
         <v>100</v>
@@ -11281,7 +11255,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ HB   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="179" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A179" s="11" t="str">
         <f t="shared" si="2"/>
         <v>378</v>
@@ -11318,7 +11292,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="180" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A180" s="11" t="str">
         <f t="shared" si="2"/>
         <v>058</v>
@@ -11358,7 +11332,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="181" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A181" s="11" t="str">
         <f t="shared" si="2"/>
         <v>058</v>
@@ -11398,7 +11372,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="182" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A182" s="11" t="str">
         <f t="shared" si="2"/>
         <v>067</v>
@@ -11438,7 +11412,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="183" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A183" s="11" t="str">
         <f t="shared" si="2"/>
         <v>067</v>
@@ -11478,7 +11452,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="184" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A184" s="11" t="str">
         <f t="shared" si="2"/>
         <v>241</v>
@@ -11514,7 +11488,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ HB   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="185" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A185" s="11" t="str">
         <f t="shared" si="2"/>
         <v>099</v>
@@ -11550,7 +11524,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ HB   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="186" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A186" s="11" t="str">
         <f t="shared" si="2"/>
         <v>238</v>
@@ -11586,7 +11560,7 @@
         <v>EcoLT  0.11D - 25C - CSĐ HB   /   NEUTRAL GRAY - 2.00M</v>
       </c>
     </row>
-    <row r="187" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A187" s="11" t="str">
         <f t="shared" si="2"/>
         <v>057</v>
@@ -11626,7 +11600,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="188" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A188" s="11" t="str">
         <f t="shared" si="2"/>
         <v>304</v>
@@ -11662,7 +11636,7 @@
         <v>Regular  0.11D - 25C - CSĐ HB   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="189" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A189" s="11" t="str">
         <f t="shared" si="2"/>
         <v>225</v>
@@ -11698,7 +11672,7 @@
         <v>Regular  0.11D - 25C - CSĐ HB   /   NEUTRAL GRAY - 2.00M</v>
       </c>
     </row>
-    <row r="190" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A190" s="11" t="str">
         <f t="shared" si="2"/>
         <v>113</v>
@@ -11738,7 +11712,7 @@
         <v>Regular  0.11D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M ASICS</v>
       </c>
     </row>
-    <row r="191" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A191" s="11" t="str">
         <f t="shared" si="2"/>
         <v>057</v>
@@ -11778,7 +11752,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="192" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A192" s="11" t="str">
         <f t="shared" si="2"/>
         <v>057</v>
@@ -11818,7 +11792,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="193" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A193" s="5" t="str">
         <f t="shared" si="2"/>
         <v>057</v>
@@ -11858,7 +11832,7 @@
         <v>Ultra  0.085D - 25C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="194" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A194" s="5" t="str">
         <f t="shared" ref="A194:A257" si="3">RIGHT(B194,3)</f>
         <v>123</v>
@@ -11898,7 +11872,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="195" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A195" s="5" t="str">
         <f t="shared" si="3"/>
         <v>120</v>
@@ -11934,7 +11908,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="196" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A196" s="5" t="str">
         <f t="shared" si="3"/>
         <v>123</v>
@@ -11974,7 +11948,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="197" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A197" s="5" t="str">
         <f t="shared" si="3"/>
         <v>237</v>
@@ -12010,7 +11984,7 @@
         <v>Regular  0.11D - 25C - CSĐ HB   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="198" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A198" s="5" t="str">
         <f t="shared" si="3"/>
         <v>114</v>
@@ -12046,7 +12020,7 @@
         <v>Regular  0.11D - 25C - CSĐ HB   /   SEEDPEARL -  1.7M</v>
       </c>
     </row>
-    <row r="199" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A199" s="5" t="str">
         <f t="shared" si="3"/>
         <v>115</v>
@@ -12082,7 +12056,7 @@
         <v>Regular  0.11D - 25C - CSĐ HB   /   YELLOW -  1.7M</v>
       </c>
     </row>
-    <row r="200" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A200" s="5" t="str">
         <f t="shared" si="3"/>
         <v>142</v>
@@ -12118,7 +12092,7 @@
         <v>Regular  0.11D - 25C - NIKE   /   FOSSIL - 2.00M</v>
       </c>
     </row>
-    <row r="201" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A201" s="5" t="str">
         <f t="shared" si="3"/>
         <v>140</v>
@@ -12154,7 +12128,7 @@
         <v>Regular  0.11D - 25C - NIKE   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="202" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A202" s="5" t="str">
         <f t="shared" si="3"/>
         <v>132</v>
@@ -12190,7 +12164,7 @@
         <v>Regular  0.11D - 25C - NIKE   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="203" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A203" s="5" t="str">
         <f t="shared" si="3"/>
         <v>128</v>
@@ -12226,7 +12200,7 @@
         <v>Regular  0.11D - 25C - NIKE   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="204" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A204" s="5" t="str">
         <f t="shared" si="3"/>
         <v>141</v>
@@ -12262,7 +12236,7 @@
         <v>Regular  0.11D - 25C - NIKE   /   NEUTRAL GRAY - 2.00M</v>
       </c>
     </row>
-    <row r="205" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A205" s="5" t="str">
         <f t="shared" si="3"/>
         <v>183</v>
@@ -12298,7 +12272,7 @@
         <v>Regular  0.11D - 25C - NIKE   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="206" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A206" s="5" t="str">
         <f t="shared" si="3"/>
         <v>185</v>
@@ -12334,7 +12308,7 @@
         <v>Regular  0.11D - 25C - NIKE   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="207" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A207" s="5" t="str">
         <f t="shared" si="3"/>
         <v>123</v>
@@ -12374,7 +12348,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="208" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A208" s="5" t="str">
         <f t="shared" si="3"/>
         <v>123</v>
@@ -12414,7 +12388,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="209" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A209" s="5" t="str">
         <f t="shared" si="3"/>
         <v>129</v>
@@ -12454,7 +12428,7 @@
         <v>Regular  0.11D - 25C - Nike   /   AIR BLUE - 1.7M</v>
       </c>
     </row>
-    <row r="210" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A210" s="5" t="str">
         <f t="shared" si="3"/>
         <v>123</v>
@@ -12494,7 +12468,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="211" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A211" s="5" t="str">
         <f t="shared" si="3"/>
         <v>123</v>
@@ -12534,7 +12508,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="212" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A212" s="5" t="str">
         <f t="shared" si="3"/>
         <v>126</v>
@@ -12574,7 +12548,7 @@
         <v>Regular  0.11D - 25C - Nike   /   RED - 2.00M</v>
       </c>
     </row>
-    <row r="213" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A213" s="5" t="str">
         <f t="shared" si="3"/>
         <v>123</v>
@@ -12614,7 +12588,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="214" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A214" s="5" t="str">
         <f t="shared" si="3"/>
         <v>138</v>
@@ -12650,7 +12624,7 @@
         <v>Regular  0.11D - 25C - NIKE   /   RED - 1.47M</v>
       </c>
     </row>
-    <row r="215" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A215" s="5" t="str">
         <f t="shared" si="3"/>
         <v>302</v>
@@ -12686,7 +12660,7 @@
         <v>Regular  0.11D - 25C - NIKE   /   GREY -  1.7M</v>
       </c>
     </row>
-    <row r="216" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A216" s="5" t="str">
         <f t="shared" si="3"/>
         <v>143</v>
@@ -12722,7 +12696,7 @@
         <v>Regular  0.11D - 25C - NIKE   /   SEEDPEARL -  1.7M</v>
       </c>
     </row>
-    <row r="217" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A217" s="5" t="str">
         <f t="shared" si="3"/>
         <v>134</v>
@@ -12758,7 +12732,7 @@
         <v>Regular  0.11D - 25C - NIKE   /   YELLOW -  1.7M</v>
       </c>
     </row>
-    <row r="218" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A218" s="5" t="str">
         <f t="shared" si="3"/>
         <v>148</v>
@@ -12794,7 +12768,7 @@
         <v>Regular  0.11D - 25C - NIKE HB   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="219" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A219" s="5" t="str">
         <f t="shared" si="3"/>
         <v>147</v>
@@ -12830,7 +12804,7 @@
         <v>Regular  0.11D - 25C - NIKE HB   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="220" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A220" s="5" t="str">
         <f t="shared" si="3"/>
         <v>123</v>
@@ -12870,7 +12844,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="221" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A221" s="5" t="str">
         <f t="shared" si="3"/>
         <v>123</v>
@@ -12910,7 +12884,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="222" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A222" s="5" t="str">
         <f t="shared" si="3"/>
         <v>150</v>
@@ -12946,7 +12920,7 @@
         <v>Regular  0.11D - 25C - NIKE HB   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="223" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A223" s="5" t="str">
         <f t="shared" si="3"/>
         <v>151</v>
@@ -12982,7 +12956,7 @@
         <v>Regular  0.11D - 25C - NIKE HB   /   YELLOW - 1.47M</v>
       </c>
     </row>
-    <row r="224" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A224" s="5" t="str">
         <f t="shared" si="3"/>
         <v>146</v>
@@ -13018,7 +12992,7 @@
         <v>Regular  0.11D - 25C - NIKE HB   /   AIR BLUE -  1.7M</v>
       </c>
     </row>
-    <row r="225" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A225" s="5" t="str">
         <f t="shared" si="3"/>
         <v>295</v>
@@ -13054,7 +13028,7 @@
         <v>Regular  0.11D - 25C - NIKE HB   /   GREY -  1.7M</v>
       </c>
     </row>
-    <row r="226" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A226" s="5" t="str">
         <f t="shared" si="3"/>
         <v>152</v>
@@ -13090,7 +13064,7 @@
         <v>Regular  0.11D - 25C - NIKE HB   /   SEEDPEARL -  1.7M</v>
       </c>
     </row>
-    <row r="227" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A227" s="5" t="str">
         <f t="shared" si="3"/>
         <v>145</v>
@@ -13126,7 +13100,7 @@
         <v>Regular  0.11D - 25C - NIKE HB   /   YELLOW -  1.7M</v>
       </c>
     </row>
-    <row r="228" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A228" s="5" t="str">
         <f t="shared" si="3"/>
         <v>372</v>
@@ -13162,7 +13136,7 @@
         <v>Float  0.12D - 25C - CSĐ   /   CASTLEROCK - 2.00M</v>
       </c>
     </row>
-    <row r="229" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A229" s="5" t="str">
         <f t="shared" si="3"/>
         <v>316</v>
@@ -13198,7 +13172,7 @@
         <v>Float  0.12D - 25C - CSĐ   /   BILLIARD - 2.00M</v>
       </c>
     </row>
-    <row r="230" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A230" s="5" t="str">
         <f t="shared" si="3"/>
         <v>355</v>
@@ -13238,7 +13212,7 @@
         <v>HybridPlus  0.12D - 25C - CSĐ HB   /   CASTLEROCK - 2.00M</v>
       </c>
     </row>
-    <row r="231" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A231" s="5" t="str">
         <f t="shared" si="3"/>
         <v>123</v>
@@ -13278,7 +13252,7 @@
         <v>Ultra  0.085D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="232" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A232" s="5" t="str">
         <f t="shared" si="3"/>
         <v>175</v>
@@ -13318,7 +13292,7 @@
         <v>Ultra  0.085D - 25C - Nike HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="233" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A233" s="5" t="str">
         <f t="shared" si="3"/>
         <v>175</v>
@@ -13358,7 +13332,7 @@
         <v>Ultra  0.085D - 25C - Nike HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="234" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A234" s="5" t="str">
         <f t="shared" si="3"/>
         <v>249</v>
@@ -13394,7 +13368,7 @@
         <v>HybridPlus-Recycled   0.12D - 25C - CSĐ HB   /   MINT GREEN - 1.47M</v>
       </c>
     </row>
-    <row r="235" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A235" s="5" t="str">
         <f t="shared" si="3"/>
         <v>233</v>
@@ -13430,7 +13404,7 @@
         <v>HybridPlus-Recycled   0.12D - 25C - CSĐ HB   /   MINT GREEN -  1.7M</v>
       </c>
     </row>
-    <row r="236" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A236" s="5" t="str">
         <f t="shared" si="3"/>
         <v>112</v>
@@ -13466,7 +13440,7 @@
         <v>Regular  0.12D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="237" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A237" s="5" t="str">
         <f t="shared" si="3"/>
         <v>303</v>
@@ -13502,7 +13476,7 @@
         <v>Regular  0.12D - 25C - NIKE HB   /    SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="238" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A238" s="5" t="str">
         <f t="shared" si="3"/>
         <v>269</v>
@@ -13538,7 +13512,7 @@
         <v>EcoLT  0.13D - 25C - CSĐ   /   FAIRWAY - 2.00M</v>
       </c>
     </row>
-    <row r="239" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A239" s="5" t="str">
         <f t="shared" si="3"/>
         <v>354</v>
@@ -13574,7 +13548,7 @@
         <v>EcoLT  0.13D - 25C - CSĐ   /   GREEN -  1.7M</v>
       </c>
     </row>
-    <row r="240" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A240" s="5" t="str">
         <f t="shared" si="3"/>
         <v>260</v>
@@ -13610,7 +13584,7 @@
         <v>EcoLT  0.11D - 35C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="241" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A241" s="5" t="str">
         <f t="shared" si="3"/>
         <v>037</v>
@@ -13646,7 +13620,7 @@
         <v>Regular  0.13D - 25C - CSĐ   /   BURNT SIENNA - 2.00M</v>
       </c>
     </row>
-    <row r="242" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A242" s="5" t="str">
         <f t="shared" si="3"/>
         <v>043</v>
@@ -13682,7 +13656,7 @@
         <v>Regular  0.13D - 25C - CSĐ   /   FOSSIL - 2.00M</v>
       </c>
     </row>
-    <row r="243" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A243" s="5" t="str">
         <f t="shared" si="3"/>
         <v>035</v>
@@ -13718,7 +13692,7 @@
         <v>Regular  0.13D - 25C - CSĐ   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="244" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A244" s="5" t="str">
         <f t="shared" si="3"/>
         <v>021</v>
@@ -13754,7 +13728,7 @@
         <v>Regular  0.13D - 25C - CSĐ   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="245" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A245" s="5" t="str">
         <f t="shared" si="3"/>
         <v>042</v>
@@ -13790,7 +13764,7 @@
         <v>Regular  0.13D - 25C - CSĐ   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="246" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A246" s="5" t="str">
         <f t="shared" si="3"/>
         <v>196</v>
@@ -13826,7 +13800,7 @@
         <v>Regular  0.13D - 25C - CSĐ   /   RED - 2.00M</v>
       </c>
     </row>
-    <row r="247" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A247" s="5" t="str">
         <f t="shared" si="3"/>
         <v>012</v>
@@ -13862,7 +13836,7 @@
         <v>Regular  0.13D - 25C - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="248" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A248" s="5" t="str">
         <f t="shared" si="3"/>
         <v>018</v>
@@ -13898,7 +13872,7 @@
         <v>Regular  0.13D - 25C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="249" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A249" s="5" t="str">
         <f t="shared" si="3"/>
         <v>343</v>
@@ -13938,7 +13912,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="250" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A250" s="5" t="str">
         <f t="shared" si="3"/>
         <v>350</v>
@@ -13974,7 +13948,7 @@
         <v>Regular  0.13D - 25C - CSĐ   /   NEUTRAL GRAY - 2.00M</v>
       </c>
     </row>
-    <row r="251" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A251" s="5" t="str">
         <f t="shared" si="3"/>
         <v>047</v>
@@ -14010,7 +13984,7 @@
         <v>Regular  0.13D - 25C - CSĐ   /   AIR BLUE -  1.7M</v>
       </c>
     </row>
-    <row r="252" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A252" s="5" t="str">
         <f t="shared" si="3"/>
         <v>078</v>
@@ -14050,7 +14024,7 @@
         <v>X-30  0.13D - 25C - CSĐ   /   RED - 2.00M</v>
       </c>
     </row>
-    <row r="253" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A253" s="5" t="str">
         <f t="shared" si="3"/>
         <v>240</v>
@@ -14086,7 +14060,7 @@
         <v>X-30  0.13D - 25C - CSĐ   /   CASTLEROCK - 2.00M</v>
       </c>
     </row>
-    <row r="254" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A254" s="5" t="str">
         <f t="shared" si="3"/>
         <v>227</v>
@@ -14122,7 +14096,7 @@
         <v>X-30  0.13D - 25C - CSĐ   /    SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="255" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A255" s="5" t="str">
         <f t="shared" si="3"/>
         <v>308</v>
@@ -14158,7 +14132,7 @@
         <v>X-30  0.13D - 25C - CSĐ   /   CASTLEROCK - 1.47M</v>
       </c>
     </row>
-    <row r="256" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A256" s="5" t="str">
         <f t="shared" si="3"/>
         <v>180</v>
@@ -14198,7 +14172,7 @@
         <v>EcoLT  0.13D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="257" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A257" s="5" t="str">
         <f t="shared" si="3"/>
         <v>098</v>
@@ -14234,7 +14208,7 @@
         <v>EcoLT  0.13D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="258" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A258" s="5" t="str">
         <f t="shared" ref="A258:A321" si="4">RIGHT(B258,3)</f>
         <v>200</v>
@@ -14274,7 +14248,7 @@
         <v>Ultra  0.085D - 78-90F - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="259" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A259" s="5" t="str">
         <f t="shared" si="4"/>
         <v>200</v>
@@ -14314,7 +14288,7 @@
         <v>Ultra  0.085D - 78-90F - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="260" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A260" s="5" t="str">
         <f t="shared" si="4"/>
         <v>116</v>
@@ -14350,7 +14324,7 @@
         <v>Regular  0.13D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="261" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A261" s="5" t="str">
         <f t="shared" si="4"/>
         <v>286</v>
@@ -14390,7 +14364,7 @@
         <v>Regular  0.13D - 25C - CSĐ HB   /   SEEDPEARL - 1.7M</v>
       </c>
     </row>
-    <row r="262" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A262" s="5" t="str">
         <f t="shared" si="4"/>
         <v>299</v>
@@ -14426,7 +14400,7 @@
         <v>Regular  0.13D - 25C - CSĐ HB   /    SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="263" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A263" s="5" t="str">
         <f t="shared" si="4"/>
         <v>211</v>
@@ -14462,7 +14436,7 @@
         <v>X-30  0.13D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="264" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A264" s="5" t="str">
         <f t="shared" si="4"/>
         <v>234</v>
@@ -14502,7 +14476,7 @@
         <v>X-30  0.13D - 25C - CSĐ HB   /   BROWN SUGAR - 2.00M</v>
       </c>
     </row>
-    <row r="265" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A265" s="5" t="str">
         <f t="shared" si="4"/>
         <v>029</v>
@@ -14538,7 +14512,7 @@
         <v>Regular  0.13D - 25C - CSĐ   /   AIR BLUE - 1.47M</v>
       </c>
     </row>
-    <row r="266" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A266" s="5" t="str">
         <f t="shared" si="4"/>
         <v>079</v>
@@ -14574,7 +14548,7 @@
         <v>X-35  0.145D - 25C - CSĐ   /   AMAZON - 2.00M</v>
       </c>
     </row>
-    <row r="267" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A267" s="5" t="str">
         <f t="shared" si="4"/>
         <v>081</v>
@@ -14610,7 +14584,7 @@
         <v>X-35  0.145D - 25C - CSĐ   /   FOSSIL - 2.00M</v>
       </c>
     </row>
-    <row r="268" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A268" s="5" t="str">
         <f t="shared" si="4"/>
         <v>268</v>
@@ -14646,7 +14620,7 @@
         <v>X-35  0.145D - 25C - CSĐ   /   TRUE BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="269" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A269" s="5" t="str">
         <f t="shared" si="4"/>
         <v>080</v>
@@ -14682,7 +14656,7 @@
         <v>X-35  0.145D - 25C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="270" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A270" s="5" t="str">
         <f t="shared" si="4"/>
         <v>082</v>
@@ -14718,7 +14692,7 @@
         <v>X-35  0.145D - 25C - CSĐ   /   AMAZON - 1.47M</v>
       </c>
     </row>
-    <row r="271" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A271" s="5" t="str">
         <f t="shared" si="4"/>
         <v>259</v>
@@ -14758,7 +14732,7 @@
         <v>X-35  0.145D - 25C - CSĐ HB   /   GLACIER GRAY - 2.00M</v>
       </c>
     </row>
-    <row r="272" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A272" s="5" t="str">
         <f t="shared" si="4"/>
         <v>252</v>
@@ -14794,7 +14768,7 @@
         <v>X-35  0.145D - 25C - CSĐ HB   /   AMAZON - 2.00M</v>
       </c>
     </row>
-    <row r="273" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A273" s="5" t="str">
         <f t="shared" si="4"/>
         <v>351</v>
@@ -14830,7 +14804,7 @@
         <v>X-35  0.145D - 25C - CSĐ HB   /   FOSSIL - 2.00M</v>
       </c>
     </row>
-    <row r="274" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A274" s="5" t="str">
         <f t="shared" si="4"/>
         <v>307</v>
@@ -14866,7 +14840,7 @@
         <v>X-35  0.145D - 25C - CSĐ HB   /    SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="275" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A275" s="5" t="str">
         <f t="shared" si="4"/>
         <v>289</v>
@@ -14902,7 +14876,7 @@
         <v>X-35  0.145D - 25C - CSĐ HB   /   FOSSIL -  1.7M</v>
       </c>
     </row>
-    <row r="276" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A276" s="5" t="str">
         <f t="shared" si="4"/>
         <v>229</v>
@@ -14942,7 +14916,7 @@
         <v>Ultra  0.095D - 33C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="277" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A277" s="5" t="str">
         <f t="shared" si="4"/>
         <v>229</v>
@@ -14982,7 +14956,7 @@
         <v>Ultra  0.095D - 33C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="278" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A278" s="5" t="str">
         <f t="shared" si="4"/>
         <v>338</v>
@@ -15022,7 +14996,7 @@
         <v>X-35  0.145D - 25C - CSĐ HB   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="279" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A279" s="5" t="str">
         <f t="shared" si="4"/>
         <v>076</v>
@@ -15062,7 +15036,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   BILLIARD - 2.00M</v>
       </c>
     </row>
-    <row r="280" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A280" s="5" t="str">
         <f t="shared" si="4"/>
         <v>153</v>
@@ -15098,7 +15072,7 @@
         <v>X-35  0.145D - 25C - NIKE   /   AMAZON - 2.00M</v>
       </c>
     </row>
-    <row r="281" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A281" s="5" t="str">
         <f t="shared" si="4"/>
         <v>331</v>
@@ -15134,7 +15108,7 @@
         <v>X-35  0.145D - 25C - NIKE   /   FOSSIL - 2.00M</v>
       </c>
     </row>
-    <row r="282" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A282" s="5" t="str">
         <f t="shared" si="4"/>
         <v>327</v>
@@ -15170,7 +15144,7 @@
         <v>X-35  0.145D - 25C - NIKE   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="283" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A283" s="5" t="str">
         <f t="shared" si="4"/>
         <v>305</v>
@@ -15210,7 +15184,7 @@
         <v>X-35  0.145D - 25C - Nike   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="284" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A284" s="5" t="str">
         <f t="shared" si="4"/>
         <v>244</v>
@@ -15246,7 +15220,7 @@
         <v>X-35  0.145D - 25C - NIKE HB   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="285" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A285" s="5" t="str">
         <f t="shared" si="4"/>
         <v>236</v>
@@ -15282,7 +15256,7 @@
         <v>X-35  0.145D - 25C - NIKE HB   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="286" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A286" s="5" t="str">
         <f t="shared" si="4"/>
         <v>156</v>
@@ -15322,7 +15296,7 @@
         <v>X-35  0.145D - 25C - Nike HB   /   AMAZON - 2.00M</v>
       </c>
     </row>
-    <row r="287" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A287" s="5" t="str">
         <f t="shared" si="4"/>
         <v>076</v>
@@ -15362,7 +15336,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   BILLIARD - 2.00M</v>
       </c>
     </row>
-    <row r="288" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A288" s="5" t="str">
         <f t="shared" si="4"/>
         <v>076</v>
@@ -15402,7 +15376,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   BILLIARD - 2.00M</v>
       </c>
     </row>
-    <row r="289" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A289" s="5" t="str">
         <f t="shared" si="4"/>
         <v>076</v>
@@ -15442,7 +15416,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   BILLIARD - 2.00M</v>
       </c>
     </row>
-    <row r="290" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A290" s="5" t="str">
         <f t="shared" si="4"/>
         <v>330</v>
@@ -15482,7 +15456,7 @@
         <v>X-40  0.16D - 25C - CSĐ   /   CASTLEROCK - 2.00M</v>
       </c>
     </row>
-    <row r="291" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A291" s="5" t="str">
         <f t="shared" si="4"/>
         <v>326</v>
@@ -15518,7 +15492,7 @@
         <v>X-40  0.16D - 25C - CSĐ   /   RED - 2.00M</v>
       </c>
     </row>
-    <row r="292" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A292" s="5" t="str">
         <f t="shared" si="4"/>
         <v>324</v>
@@ -15554,7 +15528,7 @@
         <v>X-40  0.16D - 25C - CSĐ   /   TRUE BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="293" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A293" s="5" t="str">
         <f t="shared" si="4"/>
         <v>292</v>
@@ -15590,7 +15564,7 @@
         <v>X-40  0.16D - 25C - CSĐ   /    NEUTRAL GRAY - 1.47M</v>
       </c>
     </row>
-    <row r="294" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A294" s="5" t="str">
         <f t="shared" si="4"/>
         <v>250</v>
@@ -15630,7 +15604,7 @@
         <v>X-40  0.16D - 25C - CSĐ   /   CASTLEROCK - 1.7M</v>
       </c>
     </row>
-    <row r="295" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A295" s="5" t="str">
         <f t="shared" si="4"/>
         <v>054</v>
@@ -15670,7 +15644,7 @@
         <v>X-40  0.16D - 25C - CSĐ   /   RED - 1.7M</v>
       </c>
     </row>
-    <row r="296" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A296" s="5" t="str">
         <f t="shared" si="4"/>
         <v>056</v>
@@ -15710,7 +15684,7 @@
         <v>X-40  0.16D - 25C - CSĐ   /   SEEDPEARL - 1.7M</v>
       </c>
     </row>
-    <row r="297" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A297" s="5" t="str">
         <f t="shared" si="4"/>
         <v>251</v>
@@ -15746,7 +15720,7 @@
         <v>X-40  0.16D - 25C - CSĐ   /   BILLIARD -  1.7M</v>
       </c>
     </row>
-    <row r="298" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A298" s="5" t="str">
         <f t="shared" si="4"/>
         <v>052</v>
@@ -15786,7 +15760,7 @@
         <v>X-40  0.16D - 25C - CSĐ   /   TRUE BLUE - 1.47M</v>
       </c>
     </row>
-    <row r="299" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A299" s="5" t="str">
         <f t="shared" si="4"/>
         <v>076</v>
@@ -15826,7 +15800,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   BILLIARD - 2.00M</v>
       </c>
     </row>
-    <row r="300" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A300" s="5" t="str">
         <f t="shared" si="4"/>
         <v>076</v>
@@ -15866,7 +15840,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   BILLIARD - 2.00M</v>
       </c>
     </row>
-    <row r="301" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A301" s="5" t="str">
         <f t="shared" si="4"/>
         <v>270</v>
@@ -15902,7 +15876,7 @@
         <v>X-40  0.16D - 25C - CSĐ   /   FOSSIL -  1.7M</v>
       </c>
     </row>
-    <row r="302" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A302" s="5" t="str">
         <f t="shared" si="4"/>
         <v>015</v>
@@ -15938,7 +15912,7 @@
         <v>Regular  0.13D - 25C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="303" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A303" s="5" t="str">
         <f t="shared" si="4"/>
         <v>337</v>
@@ -15974,7 +15948,7 @@
         <v>X-55  0.16D - 25C - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="304" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A304" s="5" t="str">
         <f t="shared" si="4"/>
         <v>179</v>
@@ -16010,7 +15984,7 @@
         <v>X-55  0.16D - 25C - CSĐ   /   RED -  1.7M</v>
       </c>
     </row>
-    <row r="305" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A305" s="5" t="str">
         <f t="shared" si="4"/>
         <v>313</v>
@@ -16050,7 +16024,7 @@
         <v>X-55  0.16D - 25C - CSĐ   /   RED - 1.47M</v>
       </c>
     </row>
-    <row r="306" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A306" s="5" t="str">
         <f t="shared" si="4"/>
         <v>318</v>
@@ -16090,7 +16064,7 @@
         <v>X-55  0.16D - 25C - CSĐ   /   RED - 2.00M</v>
       </c>
     </row>
-    <row r="307" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A307" s="5" t="str">
         <f t="shared" si="4"/>
         <v>368</v>
@@ -16126,7 +16100,7 @@
         <v>X-40  0.16D - 25C - CSĐ HB   /   CASTLEROCK - 2.00M</v>
       </c>
     </row>
-    <row r="308" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A308" s="5" t="str">
         <f t="shared" si="4"/>
         <v>310</v>
@@ -16162,7 +16136,7 @@
         <v>X-40  0.16D - 25C - CSĐ HB   /   RED - 2.00M</v>
       </c>
     </row>
-    <row r="309" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A309" s="5" t="str">
         <f t="shared" si="4"/>
         <v>328</v>
@@ -16198,7 +16172,7 @@
         <v>X-40  0.16D - 25C - CSĐ HB   /   TRUE BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="310" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A310" s="5" t="str">
         <f t="shared" si="4"/>
         <v>245</v>
@@ -16234,7 +16208,7 @@
         <v>X-40  0.16D - 25C - CSĐ HB   /   CASTLEROCK -  1.7M</v>
       </c>
     </row>
-    <row r="311" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A311" s="5" t="str">
         <f t="shared" si="4"/>
         <v>281</v>
@@ -16270,7 +16244,7 @@
         <v>X-40  0.16D - 25C - CSĐ HB   /   GREY -  1.7M</v>
       </c>
     </row>
-    <row r="312" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A312" s="5" t="str">
         <f t="shared" si="4"/>
         <v>248</v>
@@ -16310,7 +16284,7 @@
         <v>X-40  0.16D - 25C - CSĐ HB   /   RED - 1.7M</v>
       </c>
     </row>
-    <row r="313" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A313" s="5" t="str">
         <f t="shared" si="4"/>
         <v>273</v>
@@ -16350,7 +16324,7 @@
         <v>X-40  0.16D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="314" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A314" s="5" t="str">
         <f t="shared" si="4"/>
         <v>077</v>
@@ -16390,7 +16364,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="315" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A315" s="5" t="str">
         <f t="shared" si="4"/>
         <v>077</v>
@@ -16430,7 +16404,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="316" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A316" s="5" t="str">
         <f t="shared" si="4"/>
         <v>290</v>
@@ -16466,7 +16440,7 @@
         <v>X-40  0.16D - 25C - CSĐ HB   /   TRUE BLUE -  1.7M</v>
       </c>
     </row>
-    <row r="317" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A317" s="5" t="str">
         <f t="shared" si="4"/>
         <v>280</v>
@@ -16502,7 +16476,7 @@
         <v>X-40  0.16D - 25C - CSĐ HB   /   YELLOW -  1.7M</v>
       </c>
     </row>
-    <row r="318" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A318" s="5" t="str">
         <f t="shared" si="4"/>
         <v>285</v>
@@ -16538,7 +16512,7 @@
         <v>X-55  0.16D - 25C - CSĐ HB   /   FOSSIL - 1.47M</v>
       </c>
     </row>
-    <row r="319" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A319" s="5" t="str">
         <f t="shared" si="4"/>
         <v>235</v>
@@ -16578,7 +16552,7 @@
         <v>X-55  0.16D - 25C - CSĐ HB   /   FOSSIL - 1.7M</v>
       </c>
     </row>
-    <row r="320" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A320" s="5" t="str">
         <f t="shared" si="4"/>
         <v>334</v>
@@ -16618,7 +16592,7 @@
         <v>X-55  0.16D - 25C - CSĐ HB   /   FOSSIL - 2.00M</v>
       </c>
     </row>
-    <row r="321" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A321" s="5" t="str">
         <f t="shared" si="4"/>
         <v>212</v>
@@ -16658,7 +16632,7 @@
         <v>X-25  0.12D - 20C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="322" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A322" s="5" t="str">
         <f t="shared" ref="A322:A385" si="5">RIGHT(B322,3)</f>
         <v>212</v>
@@ -16698,7 +16672,7 @@
         <v>X-25  0.12D - 20C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="323" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A323" s="5" t="str">
         <f t="shared" si="5"/>
         <v>212</v>
@@ -16738,7 +16712,7 @@
         <v>X-25  0.12D - 20C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="324" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A324" s="5" t="str">
         <f t="shared" si="5"/>
         <v>192</v>
@@ -16774,7 +16748,7 @@
         <v>X-40  0.16D - 25C - NIKE   /   RED -  1.7M</v>
       </c>
     </row>
-    <row r="325" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A325" s="5" t="str">
         <f t="shared" si="5"/>
         <v>253</v>
@@ -16810,7 +16784,7 @@
         <v>X-40  0.16D - 25C - NIKE   /   TRUE BLUE -  1.7M</v>
       </c>
     </row>
-    <row r="326" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A326" s="5" t="str">
         <f t="shared" si="5"/>
         <v>221</v>
@@ -16846,7 +16820,7 @@
         <v>X-40  0.16D - 25C - NIKE HB   /   SEEDPEARL -  1.7M</v>
       </c>
     </row>
-    <row r="327" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A327" s="5" t="str">
         <f t="shared" si="5"/>
         <v>212</v>
@@ -16886,7 +16860,7 @@
         <v>X-25  0.12D - 20C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="328" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A328" s="5" t="str">
         <f t="shared" si="5"/>
         <v>117</v>
@@ -16926,7 +16900,7 @@
         <v>X-35  0.145D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="329" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A329" s="5" t="str">
         <f t="shared" si="5"/>
         <v>117</v>
@@ -16966,7 +16940,7 @@
         <v>X-35  0.145D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="330" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A330" s="5" t="str">
         <f t="shared" si="5"/>
         <v>117</v>
@@ -17006,7 +16980,7 @@
         <v>X-35  0.145D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="331" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A331" s="5" t="str">
         <f t="shared" si="5"/>
         <v>362</v>
@@ -17046,7 +17020,7 @@
         <v>X-60  0.19D - 28C - CSĐ HB   /   SEEDPEARL - 1.7M</v>
       </c>
     </row>
-    <row r="332" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A332" s="5" t="str">
         <f t="shared" si="5"/>
         <v>357</v>
@@ -17082,7 +17056,7 @@
         <v>Ultra  0.095D - 33C - CSĐ   /   RED - 2.00M</v>
       </c>
     </row>
-    <row r="333" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A333" s="5" t="str">
         <f t="shared" si="5"/>
         <v>223</v>
@@ -17118,7 +17092,7 @@
         <v>Ultra  0.095D - 33C - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="334" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A334" s="5" t="str">
         <f t="shared" si="5"/>
         <v>367</v>
@@ -17158,7 +17132,7 @@
         <v>Ultra  0.095D - 33C - CSĐ   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="335" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A335" s="5" t="str">
         <f t="shared" si="5"/>
         <v>329</v>
@@ -17198,7 +17172,7 @@
         <v>Ultra  0.095D - 33C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="336" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A336" s="5" t="str">
         <f t="shared" si="5"/>
         <v>157</v>
@@ -17238,7 +17212,7 @@
         <v>X-35  0.145D - 25C - Nike HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="337" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A337" s="5" t="str">
         <f t="shared" si="5"/>
         <v>157</v>
@@ -17278,7 +17252,7 @@
         <v>X-35  0.145D - 25C - Nike HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="338" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A338" s="5" t="str">
         <f t="shared" si="5"/>
         <v>040</v>
@@ -17314,7 +17288,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   AIR BLUE -  1.7M</v>
       </c>
     </row>
-    <row r="339" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A339" s="5" t="str">
         <f t="shared" si="5"/>
         <v>091</v>
@@ -17350,7 +17324,7 @@
         <v>EcoLT  0.11D - 35C - CSĐ   /   FOSSIL - 2.00M</v>
       </c>
     </row>
-    <row r="340" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A340" s="5" t="str">
         <f t="shared" si="5"/>
         <v>086</v>
@@ -17386,7 +17360,7 @@
         <v>EcoLT  0.11D - 35C - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="341" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A341" s="5" t="str">
         <f t="shared" si="5"/>
         <v>363</v>
@@ -17426,7 +17400,7 @@
         <v>HybridPlus  0.12D - 35C - CSĐ HB   /   MINT GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="342" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A342" s="5" t="str">
         <f t="shared" si="5"/>
         <v>092</v>
@@ -17462,7 +17436,7 @@
         <v>EcoLT  0.13D - 35C - CSĐ   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="343" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A343" s="5" t="str">
         <f t="shared" si="5"/>
         <v>090</v>
@@ -17498,7 +17472,7 @@
         <v>EcoLT  0.13D - 35C - CSĐ   /   RED - 2.00M</v>
       </c>
     </row>
-    <row r="344" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A344" s="5" t="str">
         <f t="shared" si="5"/>
         <v>013</v>
@@ -17534,7 +17508,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   AIR BLUE - 1.47M</v>
       </c>
     </row>
-    <row r="345" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A345" s="5" t="str">
         <f t="shared" si="5"/>
         <v>157</v>
@@ -17574,7 +17548,7 @@
         <v>X-35  0.145D - 25C - Nike HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="346" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A346" s="5" t="str">
         <f t="shared" si="5"/>
         <v>051</v>
@@ -17614,7 +17588,7 @@
         <v>X-40  0.16D - 25C - CSĐ   /   TRUE BLUE - 1.7M</v>
       </c>
     </row>
-    <row r="347" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A347" s="5" t="str">
         <f t="shared" si="5"/>
         <v>051</v>
@@ -17654,7 +17628,7 @@
         <v>X-40  0.16D - 25C - CSĐ   /   TRUE BLUE - 1.7M</v>
       </c>
     </row>
-    <row r="348" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A348" s="5" t="str">
         <f t="shared" si="5"/>
         <v>118</v>
@@ -17690,7 +17664,7 @@
         <v>X-40  0.16D - 25C - CSĐ HB   /   SEEDPEARL -  1.7M</v>
       </c>
     </row>
-    <row r="349" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A349" s="5" t="str">
         <f t="shared" si="5"/>
         <v>198</v>
@@ -17726,7 +17700,7 @@
         <v>X-40  0.16D - 25C - CSĐ HB   /   SEEDPEARL -  1.7M</v>
       </c>
     </row>
-    <row r="350" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A350" s="5" t="str">
         <f t="shared" si="5"/>
         <v>016</v>
@@ -17766,7 +17740,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="351" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A351" s="5" t="str">
         <f t="shared" si="5"/>
         <v>301</v>
@@ -17806,7 +17780,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   NEUTRAL GRAY - 2.00M</v>
       </c>
     </row>
-    <row r="352" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A352" s="5" t="str">
         <f t="shared" si="5"/>
         <v>046</v>
@@ -17846,7 +17820,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   RED - 1.47M</v>
       </c>
     </row>
-    <row r="353" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A353" s="5" t="str">
         <f t="shared" si="5"/>
         <v>033</v>
@@ -17886,7 +17860,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="354" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A354" s="5" t="str">
         <f t="shared" si="5"/>
         <v>353</v>
@@ -17924,7 +17898,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="355" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A355" s="5" t="str">
         <f t="shared" si="5"/>
         <v>231</v>
@@ -17960,7 +17934,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   BLACK - 2.00M</v>
       </c>
     </row>
-    <row r="356" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A356" s="5" t="str">
         <f t="shared" si="5"/>
         <v>044</v>
@@ -17996,7 +17970,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   FOSSIL - 2.00M</v>
       </c>
     </row>
-    <row r="357" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A357" s="5" t="str">
         <f t="shared" si="5"/>
         <v>005</v>
@@ -18032,7 +18006,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="358" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A358" s="5" t="str">
         <f t="shared" si="5"/>
         <v>028</v>
@@ -18068,7 +18042,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="359" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A359" s="5" t="str">
         <f t="shared" si="5"/>
         <v>020</v>
@@ -18104,7 +18078,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   RED - 2.00M</v>
       </c>
     </row>
-    <row r="360" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A360" s="5" t="str">
         <f t="shared" si="5"/>
         <v>026</v>
@@ -18140,7 +18114,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="361" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A361" s="5" t="str">
         <f t="shared" si="5"/>
         <v>319</v>
@@ -18180,7 +18154,7 @@
         <v>X-40  0.16D - 25C - Nike HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="362" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A362" s="5" t="str">
         <f t="shared" si="5"/>
         <v>105</v>
@@ -18220,7 +18194,7 @@
         <v>EcoLT  0.13D - 35C - CSĐ HB   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="363" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A363" s="5" t="str">
         <f t="shared" si="5"/>
         <v>041</v>
@@ -18256,7 +18230,7 @@
         <v>Regular  0.13D - 35C - CSĐ   /   GREEN -  1.7M</v>
       </c>
     </row>
-    <row r="364" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A364" s="5" t="str">
         <f t="shared" si="5"/>
         <v>106</v>
@@ -18296,7 +18270,7 @@
         <v>EcoLT  0.13D - 35C - CSĐ HB   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="365" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A365" s="5" t="str">
         <f t="shared" si="5"/>
         <v>102</v>
@@ -18336,7 +18310,7 @@
         <v>EcoLT  0.13D - 35C - CSĐ HB   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="366" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A366" s="5" t="str">
         <f t="shared" si="5"/>
         <v>133</v>
@@ -18372,7 +18346,7 @@
         <v>Regular  0.13D - 35C - NIKE   /   AIR BLUE -  1.7M</v>
       </c>
     </row>
-    <row r="367" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A367" s="5" t="str">
         <f t="shared" si="5"/>
         <v>210</v>
@@ -18408,7 +18382,7 @@
         <v>EcoLT  0.13D - 35C - CSĐ HB   /   BLACK - 2.00M</v>
       </c>
     </row>
-    <row r="368" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A368" s="5" t="str">
         <f t="shared" si="5"/>
         <v>101</v>
@@ -18444,7 +18418,7 @@
         <v>EcoLT  0.13D - 35C - CSĐ HB   /   FOSSIL - 2.00M</v>
       </c>
     </row>
-    <row r="369" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A369" s="5" t="str">
         <f t="shared" si="5"/>
         <v>202</v>
@@ -18480,7 +18454,7 @@
         <v>EcoLT  0.13D - 35C - CSĐ HB   /   RED - 2.00M</v>
       </c>
     </row>
-    <row r="370" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A370" s="5" t="str">
         <f t="shared" si="5"/>
         <v>312</v>
@@ -18516,7 +18490,7 @@
         <v>EcoLT  0.13D - 35C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="371" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A371" s="5" t="str">
         <f t="shared" si="5"/>
         <v>306</v>
@@ -18552,7 +18526,7 @@
         <v>EcoLT  0.13D - 35C - CSĐ HB   /   FOSSIL -  1.7M</v>
       </c>
     </row>
-    <row r="372" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A372" s="5" t="str">
         <f t="shared" si="5"/>
         <v>258</v>
@@ -18588,7 +18562,7 @@
         <v>EcoLT  0.13D - 35C - CSĐ HB   /   LIME GREEN -  1.7M</v>
       </c>
     </row>
-    <row r="373" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A373" s="5" t="str">
         <f t="shared" si="5"/>
         <v>230</v>
@@ -18624,7 +18598,7 @@
         <v>Regular  0.13D - 35C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="374" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A374" s="5" t="str">
         <f t="shared" si="5"/>
         <v>144</v>
@@ -18660,7 +18634,7 @@
         <v>Regular  0.13D - 35C - NIKE   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="375" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A375" s="5" t="str">
         <f t="shared" si="5"/>
         <v>288</v>
@@ -18696,7 +18670,7 @@
         <v>Regular  0.13D - 35C - NIKE   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="376" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A376" s="5" t="str">
         <f t="shared" si="5"/>
         <v>182</v>
@@ -18732,7 +18706,7 @@
         <v>Regular  0.13D - 35C - NIKE   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="377" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A377" s="5" t="str">
         <f t="shared" si="5"/>
         <v>136</v>
@@ -18768,7 +18742,7 @@
         <v>Regular  0.13D - 35C - NIKE   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="378" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A378" s="5" t="str">
         <f t="shared" si="5"/>
         <v>135</v>
@@ -18804,7 +18778,7 @@
         <v>Regular  0.13D - 35C - NIKE   /   AIR BLUE - 1.47M</v>
       </c>
     </row>
-    <row r="379" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A379" s="5" t="str">
         <f t="shared" si="5"/>
         <v>130</v>
@@ -18844,7 +18818,7 @@
         <v>Regular  0.13D - 35C - Nike   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="380" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A380" s="5" t="str">
         <f t="shared" si="5"/>
         <v>277</v>
@@ -18880,7 +18854,7 @@
         <v>X-35  0.145D - 25C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="381" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A381" s="5" t="str">
         <f t="shared" si="5"/>
         <v>139</v>
@@ -18916,7 +18890,7 @@
         <v>Regular  0.13D - 35C - NIKE   /   YELLOW -  1.7M</v>
       </c>
     </row>
-    <row r="382" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A382" s="5" t="str">
         <f t="shared" si="5"/>
         <v>369</v>
@@ -18956,7 +18930,7 @@
         <v>X-40  0.16D - 35C - CSĐ   /   GREY - 1.7M</v>
       </c>
     </row>
-    <row r="383" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A383" s="5" t="str">
         <f t="shared" si="5"/>
         <v>278</v>
@@ -18996,7 +18970,7 @@
         <v>X-40  0.16D - 35C - CSĐ   /   SEEDPEARL - 1.7M</v>
       </c>
     </row>
-    <row r="384" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A384" s="5" t="str">
         <f t="shared" si="5"/>
         <v>319</v>
@@ -19036,7 +19010,7 @@
         <v>X-40  0.16D - 25C - Nike HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="385" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="385" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A385" s="5" t="str">
         <f t="shared" si="5"/>
         <v>055</v>
@@ -19076,7 +19050,7 @@
         <v>X-40  0.16D - 35C - CSĐ   /   TRUE BLUE - 1.7M</v>
       </c>
     </row>
-    <row r="386" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A386" s="5" t="str">
         <f t="shared" ref="A386:A449" si="6">RIGHT(B386,3)</f>
         <v>055</v>
@@ -19116,7 +19090,7 @@
         <v>X-40  0.16D - 35C - CSĐ   /   TRUE BLUE - 1.7M</v>
       </c>
     </row>
-    <row r="387" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="387" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A387" s="5" t="str">
         <f t="shared" si="6"/>
         <v>325</v>
@@ -19156,7 +19130,7 @@
         <v>X-40  0.16D - 35C - CSĐ   /   TRUE BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="388" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="388" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A388" s="5" t="str">
         <f t="shared" si="6"/>
         <v>053</v>
@@ -19192,7 +19166,7 @@
         <v>X-40  0.16D - 35C - CSĐ   /   BILLIARD -  1.7M</v>
       </c>
     </row>
-    <row r="389" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="389" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A389" s="5" t="str">
         <f t="shared" si="6"/>
         <v>271</v>
@@ -19228,7 +19202,7 @@
         <v>X-40  0.16D - 35C - CSĐ   /   CASTLEROCK -  1.7M</v>
       </c>
     </row>
-    <row r="390" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="390" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A390" s="5" t="str">
         <f t="shared" si="6"/>
         <v>247</v>
@@ -19264,7 +19238,7 @@
         <v>X-40  0.16D - 35C - CSĐ HB   /   CASTLEROCK -  1.7M</v>
       </c>
     </row>
-    <row r="391" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="391" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A391" s="5" t="str">
         <f t="shared" si="6"/>
         <v>309</v>
@@ -19304,7 +19278,7 @@
         <v>X-40  0.16D - 35C - CSĐ HB   /   NEUTRAL GRAY - 2.00M</v>
       </c>
     </row>
-    <row r="392" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="392" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A392" s="5" t="str">
         <f t="shared" si="6"/>
         <v>279</v>
@@ -19340,7 +19314,7 @@
         <v>X-40  0.16D - 35C - CSĐ HB   /   NEUTRAL GRAY -  1.7M</v>
       </c>
     </row>
-    <row r="393" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="393" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A393" s="5" t="str">
         <f t="shared" si="6"/>
         <v>246</v>
@@ -19376,7 +19350,7 @@
         <v>X-40  0.16D - 35C - CSĐ HB   /   RED -  1.7M</v>
       </c>
     </row>
-    <row r="394" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="394" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A394" s="5" t="str">
         <f t="shared" si="6"/>
         <v>055</v>
@@ -19416,7 +19390,7 @@
         <v>X-40  0.16D - 35C - CSĐ   /   TRUE BLUE - 1.7M</v>
       </c>
     </row>
-    <row r="395" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A395" s="5" t="str">
         <f t="shared" si="6"/>
         <v>217</v>
@@ -19456,7 +19430,7 @@
         <v>X-40  0.16D - 35C - CSĐ HB   /   SEEDPEARL - 1.7M</v>
       </c>
     </row>
-    <row r="396" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="396" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A396" s="5" t="str">
         <f t="shared" si="6"/>
         <v>217</v>
@@ -19496,7 +19470,7 @@
         <v>X-40  0.16D - 35C - CSĐ HB   /   SEEDPEARL - 1.7M</v>
       </c>
     </row>
-    <row r="397" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="397" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A397" s="5" t="str">
         <f t="shared" si="6"/>
         <v>282</v>
@@ -19536,7 +19510,7 @@
         <v>X-40  0.16D - 35C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="398" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="398" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A398" s="5" t="str">
         <f t="shared" si="6"/>
         <v>155</v>
@@ -19572,7 +19546,7 @@
         <v>X-40  0.16D - 35C - NIKE   /   RED -  1.7M</v>
       </c>
     </row>
-    <row r="399" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="399" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A399" s="5" t="str">
         <f t="shared" si="6"/>
         <v>186</v>
@@ -19608,7 +19582,7 @@
         <v>X-40  0.16D - 35C - NIKE   /   SEEDPEARL -  1.7M</v>
       </c>
     </row>
-    <row r="400" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="400" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A400" s="5" t="str">
         <f t="shared" si="6"/>
         <v>336</v>
@@ -19648,7 +19622,7 @@
         <v>X-40  0.16D - 35C - Nike   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="401" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A401" s="5" t="str">
         <f t="shared" si="6"/>
         <v>154</v>
@@ -19688,7 +19662,7 @@
         <v>X-40  0.16D - 35C - Nike   /   TRUE BLUE - 1.7M</v>
       </c>
     </row>
-    <row r="402" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="402" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A402" s="5" t="str">
         <f t="shared" si="6"/>
         <v>374</v>
@@ -19728,7 +19702,7 @@
         <v>Regular  0.15D - 45C - CSĐ   /   FOSSIL - 2.00M</v>
       </c>
     </row>
-    <row r="403" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="403" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A403" s="5" t="str">
         <f t="shared" si="6"/>
         <v>255</v>
@@ -19768,7 +19742,7 @@
         <v>Regular  0.15D - 45C - CSĐ   /   GREY - 1.7M</v>
       </c>
     </row>
-    <row r="404" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="404" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A404" s="5" t="str">
         <f t="shared" si="6"/>
         <v>275</v>
@@ -19808,7 +19782,7 @@
         <v>Regular  0.15D - 45C - CSĐ   /   RED - 1.7M</v>
       </c>
     </row>
-    <row r="405" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="405" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A405" s="5" t="str">
         <f t="shared" si="6"/>
         <v>298</v>
@@ -19844,7 +19818,7 @@
         <v>Regular  0.15D - 45C - CSĐ   /   AIR BLUE -  1.7M</v>
       </c>
     </row>
-    <row r="406" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="406" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A406" s="5" t="str">
         <f t="shared" si="6"/>
         <v>287</v>
@@ -19880,7 +19854,7 @@
         <v>Regular  0.15D - 45C - CSĐ   /   YELLOW - 1.7M</v>
       </c>
     </row>
-    <row r="407" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="407" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A407" s="5" t="str">
         <f t="shared" si="6"/>
         <v>048</v>
@@ -19916,7 +19890,7 @@
         <v>Regular  0.15D - 45C - CSĐ   /   (ROCKPORT) -  1.7M</v>
       </c>
     </row>
-    <row r="408" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="408" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A408" s="5" t="str">
         <f t="shared" si="6"/>
         <v>320</v>
@@ -19952,7 +19926,7 @@
         <v>Regular  0.15D - 45C - CSĐ   /   AIR BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="409" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="409" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A409" s="5" t="str">
         <f t="shared" si="6"/>
         <v>266</v>
@@ -19988,7 +19962,7 @@
         <v>Regular  0.15D - 45C - CSĐ   /   BLACK -  1.7M</v>
       </c>
     </row>
-    <row r="410" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="410" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A410" s="5" t="str">
         <f t="shared" si="6"/>
         <v>257</v>
@@ -20024,7 +19998,7 @@
         <v>Regular  0.15D - 45C - CSĐ   /   FOSSIL -  1.7M</v>
       </c>
     </row>
-    <row r="411" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="411" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A411" s="5" t="str">
         <f t="shared" si="6"/>
         <v>256</v>
@@ -20060,7 +20034,7 @@
         <v>Regular  0.15D - 45C - CSĐ   /   LIME GREEN -  1.7M</v>
       </c>
     </row>
-    <row r="412" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="412" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A412" s="5" t="str">
         <f t="shared" si="6"/>
         <v>291</v>
@@ -20096,7 +20070,7 @@
         <v>Regular  0.15D - 45C - CSĐ   /   NEUTRAL GRAY -  1.7M</v>
       </c>
     </row>
-    <row r="413" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="413" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A413" s="5" t="str">
         <f t="shared" si="6"/>
         <v>254</v>
@@ -20132,7 +20106,7 @@
         <v>Regular  0.15D - 45C - CSĐ   /   SEEDPEARL -  1.7M</v>
       </c>
     </row>
-    <row r="414" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="414" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A414" s="5" t="str">
         <f t="shared" si="6"/>
         <v>216</v>
@@ -20168,7 +20142,7 @@
         <v>Nike  0.15D - 45C - NIKE   /   AIR BLUE -  1.7M</v>
       </c>
     </row>
-    <row r="415" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="415" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A415" s="5" t="str">
         <f t="shared" si="6"/>
         <v>215</v>
@@ -20204,7 +20178,7 @@
         <v>Nike  0.15D - 45C - NIKE   /   SEEDPEARL -  1.7M</v>
       </c>
     </row>
-    <row r="416" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="416" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A416" s="5" t="str">
         <f t="shared" si="6"/>
         <v>214</v>
@@ -20240,7 +20214,7 @@
         <v>Nike  0.15D - 45C - NIKE   /   YELLOW -  1.7M</v>
       </c>
     </row>
-    <row r="417" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="417" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A417" s="5" t="str">
         <f t="shared" si="6"/>
         <v>296</v>
@@ -20276,7 +20250,7 @@
         <v>Regular  0.15D - 45C - NIKE   /   GREY -  1.7M</v>
       </c>
     </row>
-    <row r="418" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="418" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A418" s="5" t="str">
         <f t="shared" si="6"/>
         <v>371</v>
@@ -20312,7 +20286,7 @@
         <v>SloMo  0.085D - 5-10C - CSĐ   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="419" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="419" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A419" s="5" t="str">
         <f t="shared" si="6"/>
         <v>204</v>
@@ -20348,7 +20322,7 @@
         <v>Ultra  0.085D - 5-10C - CSĐ   /   BURNT SIENNA - 2.00M</v>
       </c>
     </row>
-    <row r="420" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="420" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A420" s="5" t="str">
         <f t="shared" si="6"/>
         <v>205</v>
@@ -20384,7 +20358,7 @@
         <v>Ultra  0.085D - 5-10C - CSĐ   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="421" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="421" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A421" s="5" t="str">
         <f t="shared" si="6"/>
         <v>203</v>
@@ -20420,7 +20394,7 @@
         <v>Ultra  0.085D - 5-10C - CSĐ   /   RED - 2.00M</v>
       </c>
     </row>
-    <row r="422" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="422" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A422" s="5" t="str">
         <f t="shared" si="6"/>
         <v>361</v>
@@ -20456,7 +20430,7 @@
         <v>X-40  0.16D - 25C - CSĐ   /   AIR BLUE -  1.7M</v>
       </c>
     </row>
-    <row r="423" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="423" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A423" s="5" t="str">
         <f t="shared" si="6"/>
         <v>206</v>
@@ -20492,7 +20466,7 @@
         <v>Ultra  0.085D - 5-10C - CSĐ   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="424" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="424" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A424" s="5" t="str">
         <f t="shared" si="6"/>
         <v>201</v>
@@ -20528,7 +20502,7 @@
         <v>Ultra  0.085D - 5-10C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="425" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="425" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A425" s="5" t="str">
         <f t="shared" si="6"/>
         <v>199</v>
@@ -20564,7 +20538,7 @@
         <v>Ultra  0.085D - 5-10C - CSĐ HB   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="426" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="426" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A426" s="5" t="str">
         <f t="shared" si="6"/>
         <v>197</v>
@@ -20604,7 +20578,7 @@
         <v>Ultra  0.085D - 5-10C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="427" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="427" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A427" s="5" t="str">
         <f t="shared" si="6"/>
         <v>218</v>
@@ -20640,7 +20614,7 @@
         <v>Ultra  0.085D - 5-10C - NIKE   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="428" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="428" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A428" s="5" t="str">
         <f t="shared" si="6"/>
         <v>315</v>
@@ -20676,7 +20650,7 @@
         <v>Regular  0.11D - 5-10C - CSĐ   /   LIME GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="429" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="429" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A429" s="5" t="str">
         <f t="shared" si="6"/>
         <v>208</v>
@@ -20712,7 +20686,7 @@
         <v>Regular  0.11D - 5-10C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="430" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="430" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A430" s="5" t="str">
         <f t="shared" si="6"/>
         <v>242</v>
@@ -20752,7 +20726,7 @@
         <v>Regular  0.11D - 5-10C - CSĐ   /   GREY - 2.00M</v>
       </c>
     </row>
-    <row r="431" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="431" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A431" s="5" t="str">
         <f t="shared" si="6"/>
         <v>222</v>
@@ -20788,7 +20762,7 @@
         <v>Regular  0.11D - 5-10C - CSĐ   /   YELLOW - 1.47M</v>
       </c>
     </row>
-    <row r="432" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="432" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A432" s="5" t="str">
         <f t="shared" si="6"/>
         <v>261</v>
@@ -20824,7 +20798,7 @@
         <v>Regular  0.11D - 5-10C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="433" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="433" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A433" s="5" t="str">
         <f t="shared" si="6"/>
         <v>226</v>
@@ -20864,7 +20838,7 @@
         <v>Regular  0.16D - 51C - CSĐ   /   GREY - 1.7M</v>
       </c>
     </row>
-    <row r="434" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="434" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A434" s="5" t="str">
         <f t="shared" si="6"/>
         <v>314</v>
@@ -20904,7 +20878,7 @@
         <v>Regular  0.16D - 51C - CSĐ   /   NEUTRAL GRAY - 1.7M</v>
       </c>
     </row>
-    <row r="435" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="435" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A435" s="5" t="str">
         <f t="shared" si="6"/>
         <v>335</v>
@@ -20940,7 +20914,7 @@
         <v>Regular  0.16D - 51C - CSĐ   /   SEEDPEARL -  1.7M</v>
       </c>
     </row>
-    <row r="436" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="436" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A436" s="5" t="str">
         <f t="shared" si="6"/>
         <v>322</v>
@@ -20976,7 +20950,7 @@
         <v>Regular  0.16D - 51C - CSĐ   /   BLACK -  1.7M</v>
       </c>
     </row>
-    <row r="437" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="437" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A437" s="5" t="str">
         <f t="shared" si="6"/>
         <v>386</v>
@@ -21012,7 +20986,7 @@
         <v>Impressions  0.15D - 70-80C - CSĐ   /   SEEDPEARL -  1.7M</v>
       </c>
     </row>
-    <row r="438" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="438" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A438" s="5" t="str">
         <f t="shared" si="6"/>
         <v>384</v>
@@ -21048,7 +21022,7 @@
         <v>Impressions SEEDPEARL  0.15D - 70-80C - CSĐ   /   SEEDPEARL - 1.7M</v>
       </c>
     </row>
-    <row r="439" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="439" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A439" s="5" t="str">
         <f t="shared" si="6"/>
         <v>284</v>
@@ -21084,7 +21058,7 @@
         <v>Lazy  0.15D - 72-78C - CSĐ   /   YELLOW - 1.47M</v>
       </c>
     </row>
-    <row r="440" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="440" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A440" s="5" t="str">
         <f t="shared" si="6"/>
         <v>293</v>
@@ -21120,7 +21094,7 @@
         <v>Lazy  0.15D - 72-78C - CSĐ   /   SEEDPEARL -  1.7M</v>
       </c>
     </row>
-    <row r="441" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="441" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A441" s="5" t="str">
         <f t="shared" si="6"/>
         <v>274</v>
@@ -21156,7 +21130,7 @@
         <v>Lazy  0.15D - 72-78C - CSĐ   /   YELLOW -  1.7M</v>
       </c>
     </row>
-    <row r="442" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="442" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A442" s="5" t="str">
         <f t="shared" si="6"/>
         <v>333</v>
@@ -21192,7 +21166,7 @@
         <v>Ultra  0.085D - 78-90C - CSĐ   /   YELLOW - 2.00M</v>
       </c>
     </row>
-    <row r="443" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="443" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A443" s="5" t="str">
         <f t="shared" si="6"/>
         <v>228</v>
@@ -21228,7 +21202,7 @@
         <v>Ultra  0.085D - 78-90C - CSĐ   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="444" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="444" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A444" s="5" t="str">
         <f t="shared" si="6"/>
         <v>323</v>
@@ -21264,7 +21238,7 @@
         <v>Ultra-Nike  0.085D - 78-90C - NIKE   /   YELLOW -  1.7M</v>
       </c>
     </row>
-    <row r="445" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="445" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A445" s="5" t="str">
         <f t="shared" si="6"/>
         <v>217</v>
@@ -21304,7 +21278,7 @@
         <v>X-40  0.16D - 35C - CSĐ HB   /   SEEDPEARL - 1.7M</v>
       </c>
     </row>
-    <row r="446" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="446" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A446" s="5" t="str">
         <f t="shared" si="6"/>
         <v>347</v>
@@ -21344,7 +21318,7 @@
         <v>X-55  0.16D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="447" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="447" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A447" s="5" t="str">
         <f t="shared" si="6"/>
         <v>262</v>
@@ -21384,7 +21358,7 @@
         <v>Ultra  0.085D - 78-90F - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="448" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="448" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A448" s="11" t="str">
         <f t="shared" si="6"/>
         <v>385</v>
@@ -21418,7 +21392,7 @@
         <v>IMPRESSION  0.15D - 70-80C - NIKE   /   TAWNY PORT - 1.7M</v>
       </c>
     </row>
-    <row r="449" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="449" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A449" s="11" t="str">
         <f t="shared" si="6"/>
         <v>382</v>
@@ -21456,7 +21430,7 @@
         <v>Regular  0.16D - 51C - CSĐ   /   FOSSIL - 1.7M</v>
       </c>
     </row>
-    <row r="450" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="450" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A450" s="11" t="str">
         <f t="shared" ref="A450:A454" si="7">RIGHT(B450,3)</f>
         <v>347</v>
@@ -21496,7 +21470,7 @@
         <v>X-55  0.16D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="451" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="451" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A451" s="11" t="str">
         <f t="shared" si="7"/>
         <v>347</v>
@@ -21536,7 +21510,7 @@
         <v>X-55  0.16D - 25C - CSĐ HB   /   SEEDPEARL - 2.00M</v>
       </c>
     </row>
-    <row r="452" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="452" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A452" s="5" t="str">
         <f t="shared" si="7"/>
         <v>392</v>
@@ -21574,7 +21548,7 @@
         <v>X-40  0.16D - 35C - NIKE   /   TRUE BLUE - 2.00M</v>
       </c>
     </row>
-    <row r="453" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="453" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A453" s="11" t="str">
         <f t="shared" si="7"/>
         <v>391</v>
@@ -21612,7 +21586,7 @@
         <v>HybridPlus  0.12D - 25C - CSĐ HB   /   COLORO - 2.00M</v>
       </c>
     </row>
-    <row r="454" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="454" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A454" s="11" t="str">
         <f t="shared" si="7"/>
         <v>393</v>
@@ -21650,7 +21624,7 @@
         <v>X-25  0.12D - 20C - CSĐ   /   GREEN - 2.00M</v>
       </c>
     </row>
-    <row r="455" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="455" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A455" s="11" t="str">
         <f>RIGHT(B455,3)</f>
         <v>389</v>
@@ -21686,7 +21660,7 @@
         <v>FLOAT  0.12D - 21C - NIKE   /   BLUE ATOLL - 2.00M</v>
       </c>
     </row>
-    <row r="456" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="456" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A456" s="11" t="str">
         <f>RIGHT(B456,3)</f>
         <v>388</v>
@@ -21722,7 +21696,7 @@
         <v>ULTRA  0.085D - 25C - NIKE   /   SEEDPEARL - 1.47M</v>
       </c>
     </row>
-    <row r="457" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="457" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A457" s="11" t="str">
         <f>RIGHT(B457,3)</f>
         <v>385</v>
@@ -21758,7 +21732,7 @@
         <v>IMPRESSION  0.15D - 70-80C - NIKE   /   TAWNY PORT - 1.7M</v>
       </c>
     </row>
-    <row r="458" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="458" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A458" s="11" t="str">
         <f>RIGHT(B458,3)</f>
         <v>385</v>

</xml_diff>